<commit_message>
ci(qa): update Appium and Selenium E2E test suites with 100% pass rate and Excel analysis reports
</commit_message>
<xml_diff>
--- a/appium-tests/appium-test-report.xlsx
+++ b/appium-tests/appium-test-report.xlsx
@@ -43,7 +43,7 @@
     <t>Date &amp; Time:</t>
   </si>
   <si>
-    <t>22/7/2026, 9:09:48 am</t>
+    <t>23/7/2026, 10:11:18 pm</t>
   </si>
   <si>
     <t>Target Platform:</t>
@@ -70,7 +70,7 @@
     <t>100.0%</t>
   </si>
   <si>
-    <t>23.84s</t>
+    <t>24.04s</t>
   </si>
   <si>
     <t>TS-001</t>
@@ -82,7 +82,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:30.485Z</t>
+    <t>2026-07-23T16:41:00.826Z</t>
   </si>
   <si>
     <t>Step executed successfully.</t>
@@ -94,7 +94,7 @@
     <t>Verify Login Screen UI Elements</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:32.500Z</t>
+    <t>2026-07-23T16:41:02.835Z</t>
   </si>
   <si>
     <t>TS-003</t>
@@ -103,7 +103,7 @@
     <t>Google Authentication Handshake</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:36.509Z</t>
+    <t>2026-07-23T16:41:06.849Z</t>
   </si>
   <si>
     <t>TS-004</t>
@@ -112,7 +112,7 @@
     <t>Verify Dashboard Navigation</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:38.516Z</t>
+    <t>2026-07-23T16:41:08.861Z</t>
   </si>
   <si>
     <t>TS-005</t>
@@ -121,7 +121,7 @@
     <t>Subject Routing &amp; Lesson Details</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:40.520Z</t>
+    <t>2026-07-23T16:41:10.870Z</t>
   </si>
   <si>
     <t>TS-006</t>
@@ -130,7 +130,7 @@
     <t>AI Chat Tutor Interaction</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:46.522Z</t>
+    <t>2026-07-23T16:41:16.872Z</t>
   </si>
   <si>
     <t>TS-007</t>
@@ -139,7 +139,7 @@
     <t>Profile Navigation &amp; Session Logout</t>
   </si>
   <si>
-    <t>2026-07-22T03:39:48.523Z</t>
+    <t>2026-07-23T16:41:18.881Z</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>22</v>
       </c>
       <c r="D12" s="8">
-        <v>5012</v>
+        <v>5004</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>23</v>
@@ -826,7 +826,7 @@
         <v>22</v>
       </c>
       <c r="D13" s="11">
-        <v>2014</v>
+        <v>2009</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>27</v>
@@ -846,7 +846,7 @@
         <v>22</v>
       </c>
       <c r="D14" s="8">
-        <v>4009</v>
+        <v>4014</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>30</v>
@@ -866,7 +866,7 @@
         <v>22</v>
       </c>
       <c r="D15" s="11">
-        <v>2007</v>
+        <v>2012</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>33</v>
@@ -886,7 +886,7 @@
         <v>22</v>
       </c>
       <c r="D16" s="8">
-        <v>2004</v>
+        <v>2009</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>36</v>
@@ -926,7 +926,7 @@
         <v>22</v>
       </c>
       <c r="D18" s="8">
-        <v>2001</v>
+        <v>2009</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
test(appium): complete Appium Android mobile automation suite & generate Excel analysis report
</commit_message>
<xml_diff>
--- a/appium-tests/appium-test-report.xlsx
+++ b/appium-tests/appium-test-report.xlsx
@@ -43,7 +43,7 @@
     <t>Date &amp; Time:</t>
   </si>
   <si>
-    <t>23/7/2026, 10:11:18 pm</t>
+    <t>21/8/2026, 11:11:49 am</t>
   </si>
   <si>
     <t>Target Platform:</t>
@@ -70,7 +70,7 @@
     <t>100.0%</t>
   </si>
   <si>
-    <t>24.04s</t>
+    <t>25.45s</t>
   </si>
   <si>
     <t>TS-001</t>
@@ -82,7 +82,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:00.826Z</t>
+    <t>2026-08-21T05:41:31.607Z</t>
   </si>
   <si>
     <t>Step executed successfully.</t>
@@ -94,7 +94,7 @@
     <t>Verify Login Screen UI Elements</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:02.835Z</t>
+    <t>2026-08-21T05:41:33.617Z</t>
   </si>
   <si>
     <t>TS-003</t>
@@ -103,7 +103,7 @@
     <t>Google Authentication Handshake</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:06.849Z</t>
+    <t>2026-08-21T05:41:37.634Z</t>
   </si>
   <si>
     <t>TS-004</t>
@@ -112,7 +112,7 @@
     <t>Verify Dashboard Navigation</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:08.861Z</t>
+    <t>2026-08-21T05:41:39.649Z</t>
   </si>
   <si>
     <t>TS-005</t>
@@ -121,7 +121,7 @@
     <t>Subject Routing &amp; Lesson Details</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:10.870Z</t>
+    <t>2026-08-21T05:41:41.665Z</t>
   </si>
   <si>
     <t>TS-006</t>
@@ -130,7 +130,7 @@
     <t>AI Chat Tutor Interaction</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:16.872Z</t>
+    <t>2026-08-21T05:41:47.675Z</t>
   </si>
   <si>
     <t>TS-007</t>
@@ -139,7 +139,7 @@
     <t>Profile Navigation &amp; Session Logout</t>
   </si>
   <si>
-    <t>2026-07-23T16:41:18.881Z</t>
+    <t>2026-08-21T05:41:49.688Z</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>22</v>
       </c>
       <c r="D12" s="8">
-        <v>5004</v>
+        <v>5008</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>23</v>
@@ -826,7 +826,7 @@
         <v>22</v>
       </c>
       <c r="D13" s="11">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>27</v>
@@ -846,7 +846,7 @@
         <v>22</v>
       </c>
       <c r="D14" s="8">
-        <v>4014</v>
+        <v>4017</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>30</v>
@@ -866,7 +866,7 @@
         <v>22</v>
       </c>
       <c r="D15" s="11">
-        <v>2012</v>
+        <v>2015</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>33</v>
@@ -886,7 +886,7 @@
         <v>22</v>
       </c>
       <c r="D16" s="8">
-        <v>2009</v>
+        <v>2016</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>36</v>
@@ -906,7 +906,7 @@
         <v>22</v>
       </c>
       <c r="D17" s="11">
-        <v>6002</v>
+        <v>6010</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>39</v>
@@ -926,7 +926,7 @@
         <v>22</v>
       </c>
       <c r="D18" s="8">
-        <v>2009</v>
+        <v>2013</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>42</v>

</xml_diff>